<commit_message>
v18.12: re-fit potential on regulatory scope changes, Monte Carlo above 3 years; oracle refreshed; TS port
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01H4KMmzfQcyqrFUJptihnsX
</commit_message>
<xml_diff>
--- a/app/fixtures/xlsx/xl-reg.xlsx
+++ b/app/fixtures/xlsx/xl-reg.xlsx
@@ -6469,7 +6469,7 @@
         <v>5</v>
       </c>
       <c r="B2" s="2">
-        <v>75</v>
+        <v>46</v>
       </c>
       <c r="C2" s="3">
         <v>10</v>
@@ -27537,16 +27537,16 @@
         <v>2.99</v>
       </c>
       <c r="C2">
-        <v>1.19</v>
+        <v>1.76</v>
       </c>
       <c r="D2">
-        <v>1.8</v>
+        <v>1.23</v>
       </c>
       <c r="E2">
-        <v>-1.8</v>
+        <v>-1.23</v>
       </c>
       <c r="F2">
-        <v>60</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -27557,16 +27557,16 @@
         <v>8.15</v>
       </c>
       <c r="C3">
-        <v>2.53</v>
+        <v>4.29</v>
       </c>
       <c r="D3">
-        <v>5.63</v>
+        <v>3.86</v>
       </c>
       <c r="E3">
-        <v>-5.63</v>
+        <v>-3.86</v>
       </c>
       <c r="F3">
-        <v>69</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -27577,16 +27577,16 @@
         <v>3.86</v>
       </c>
       <c r="C4">
-        <v>1.23</v>
+        <v>2.05</v>
       </c>
       <c r="D4">
-        <v>2.62</v>
+        <v>1.8</v>
       </c>
       <c r="E4">
-        <v>-2.62</v>
+        <v>-1.8</v>
       </c>
       <c r="F4">
-        <v>68</v>
+        <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -27597,10 +27597,10 @@
         <v>15</v>
       </c>
       <c r="C5">
-        <v>4.95</v>
+        <v>8.1</v>
       </c>
       <c r="D5">
-        <v>10.05</v>
+        <v>6.9</v>
       </c>
       <c r="E5" t="s">
         <v>25</v>
@@ -29749,10 +29749,10 @@
         <v>5</v>
       </c>
       <c r="E3" s="3">
-        <v>829.1</v>
+        <v>569.3</v>
       </c>
       <c r="F3" s="3">
-        <v>1990</v>
+        <v>1366</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -29769,10 +29769,10 @@
         <v>15</v>
       </c>
       <c r="E4" s="3">
-        <v>1105.5</v>
+        <v>759</v>
       </c>
       <c r="F4" s="3">
-        <v>7960</v>
+        <v>5465</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -29789,10 +29789,10 @@
         <v>75</v>
       </c>
       <c r="E5" s="3">
-        <v>829.1</v>
+        <v>569.3</v>
       </c>
       <c r="F5" s="3">
-        <v>29849</v>
+        <v>20493</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>